<commit_message>
updated example data with new column.
</commit_message>
<xml_diff>
--- a/example_data/nodes/nodes.xlsx
+++ b/example_data/nodes/nodes.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="14">
   <si>
     <t xml:space="preserve">node</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t xml:space="preserve">demand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">representative_node</t>
   </si>
   <si>
     <t xml:space="preserve">elec</t>
@@ -178,7 +181,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -205,6 +208,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -414,7 +421,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.56"/>
@@ -422,6 +429,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="21.17"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -440,84 +448,99 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>7</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="F2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="7"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="C4" s="6" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>9</v>
-      </c>
+      <c r="D4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="7"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="n">
+      <c r="A5" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="7"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="13"/>
+      <c r="C7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>9</v>
-      </c>
+      <c r="F7" s="7"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F7" type="list">
+      <formula1>"X"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Support for new nodes.xlsx.
</commit_message>
<xml_diff>
--- a/example_data/nodes/nodes.xlsx
+++ b/example_data/nodes/nodes.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="14">
   <si>
     <t xml:space="preserve">node</t>
   </si>
@@ -31,7 +31,7 @@
     <t xml:space="preserve">alternative_name</t>
   </si>
   <si>
-    <t xml:space="preserve">balance_type</t>
+    <t xml:space="preserve">free_node</t>
   </si>
   <si>
     <t xml:space="preserve">demand</t>
@@ -53,9 +53,6 @@
   </si>
   <si>
     <t xml:space="preserve">market</t>
-  </si>
-  <si>
-    <t xml:space="preserve">balance_type_none</t>
   </si>
   <si>
     <t xml:space="preserve">heat</t>
@@ -498,7 +495,7 @@
         <v>7</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F4" s="7"/>
     </row>
@@ -507,13 +504,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>9</v>
@@ -524,20 +521,20 @@
         <v>2</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F7" s="7"/>
     </row>

</xml_diff>